<commit_message>
sync before new mac
</commit_message>
<xml_diff>
--- a/Restaurant Management/results/BHB_Kingsville_sorted_Kingsville_Payroll.xlsx
+++ b/Restaurant Management/results/BHB_Kingsville_sorted_Kingsville_Payroll.xlsx
@@ -495,10 +495,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.74</v>
+        <v>37.31</v>
       </c>
     </row>
     <row r="3">
@@ -509,19 +506,19 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SERVER</t>
+          <t>BAR</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>4.61</v>
+        <v>13.18</v>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>13</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>13</v>
+        <v>87.76000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -532,44 +529,40 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BAR</t>
+          <t>SERVER</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>5.4</v>
+        <v>10.13</v>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>65</v>
+        <v>126.39</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>65</v>
+        <v>126.39</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Alyssa Rodriguez</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>HOST</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>8.56</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="n">
-        <v>20.11</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>20.11</v>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Alexandra Perez</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="F5" t="n">
+        <v>91.34999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>91.34999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -584,125 +577,122 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>31.44</v>
+        <v>25.47</v>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>237.84</v>
+        <v>173.08</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>237.84</v>
+        <v>173.08</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Arnold Ramirez</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>General Manager</t>
-        </is>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Alyssa Rodriguez</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>HOST</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>14.53</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Arturo Orozco</t>
+          <t>Arnold Ramirez</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Kitchen</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>21.83</v>
+          <t>General Manager</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Austin Barnes</t>
+          <t>Arturo Orozco</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>SERVER</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.84</v>
-      </c>
-      <c r="F9" t="n">
-        <v>252.59</v>
-      </c>
-      <c r="G9" t="n">
-        <v>252.59</v>
+        <v>17.85</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
+          <t>Austin Barnes</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F10" t="n">
+        <v>39.18</v>
+      </c>
+      <c r="G10" t="n">
+        <v>39.18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
           <t>Bailee Pena</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>33.71</v>
-      </c>
-      <c r="F10" t="n">
-        <v>229.35</v>
-      </c>
-      <c r="G10" t="n">
-        <v>229.35</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>34.07</v>
+      </c>
+      <c r="F11" t="n">
+        <v>253.05</v>
+      </c>
+      <c r="G11" t="n">
+        <v>253.05</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Blaine Roberson</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>13.31</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="n">
-        <v>290.5</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>290.5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Blaine Roberson</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>MANAGER</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -716,13 +706,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9.949999999999999</v>
+        <v>6.09</v>
       </c>
       <c r="F13" t="n">
-        <v>109.5</v>
+        <v>153.97</v>
       </c>
       <c r="G13" t="n">
-        <v>109.5</v>
+        <v>153.97</v>
       </c>
     </row>
     <row r="14">
@@ -737,73 +727,73 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.74</v>
+        <v>34.08</v>
       </c>
       <c r="F14" t="n">
-        <v>174.43</v>
+        <v>322.62</v>
       </c>
       <c r="G14" t="n">
-        <v>174.43</v>
+        <v>322.62</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Clarissa Cantu</t>
+          <t>Cameron Allen</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>SERVER</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>36.41</v>
-      </c>
-      <c r="F15" t="n">
-        <v>322.16</v>
-      </c>
-      <c r="G15" t="n">
-        <v>322.16</v>
+        <v>25.06</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Dominique Zamora</t>
+          <t>Christopher Campos</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>MANAGER</t>
-        </is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>36.17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Emileigh Salinas</t>
+          <t>Clarissa Cantu</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>BAR</t>
+          <t>SERVER</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25.56</v>
+        <v>40</v>
+      </c>
+      <c r="D17" t="n">
+        <v>6.51</v>
       </c>
       <c r="F17" t="n">
-        <v>342.7</v>
+        <v>325.43</v>
       </c>
       <c r="G17" t="n">
-        <v>342.7</v>
+        <v>325.43</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Felicity Alaniz</t>
+          <t>David Barraza</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -812,19 +802,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>12.92</v>
-      </c>
-      <c r="F18" t="n">
-        <v>150.03</v>
-      </c>
-      <c r="G18" t="n">
-        <v>150.03</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Gina Galvan</t>
+          <t>David Hernandez</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -833,49 +817,40 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>11.56</v>
+        <v>23.98</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Hailey Nunn</t>
+          <t>Dominique Zamora</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>20.93</v>
-      </c>
-      <c r="F20" t="n">
-        <v>223.83</v>
-      </c>
-      <c r="G20" t="n">
-        <v>223.83</v>
+          <t>MANAGER</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Heilyn Julissa Diaz</t>
+          <t>Elizabeth Williams</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>HOST</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>36.49</v>
+        <v>4.88</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Indira Garcia</t>
+          <t>Emileigh Salinas</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -884,161 +859,160 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.14</v>
+        <v>29.07</v>
       </c>
       <c r="F22" t="n">
-        <v>215.2</v>
+        <v>263.12</v>
       </c>
       <c r="G22" t="n">
-        <v>215.2</v>
+        <v>263.12</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Isabel Garcia</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>17.09</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="n">
-        <v>212.28</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>212.28</v>
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Felicity Alaniz</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="E23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F23" t="n">
+        <v>51.84</v>
+      </c>
+      <c r="G23" t="n">
+        <v>61.84</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Isabel Garcia</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Customer Service Liaison</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>9.609999999999999</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Gilbert Garza</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>38.36</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Isabella Salinas</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="n">
-        <v>62.76</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>62.76</v>
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Hailey Nunn</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="F25" t="n">
+        <v>240.09</v>
+      </c>
+      <c r="G25" t="n">
+        <v>240.09</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Isabella Salinas</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="n">
-        <v>281.41</v>
-      </c>
-      <c r="G26" s="3" t="n">
-        <v>281.41</v>
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Heilyn Julissa Diaz</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>40</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3.86</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>J'Elle Longoria</t>
+          <t>Indira Garcia</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>SERVER</t>
+          <t>BAR</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>29.66</v>
+        <v>27.39</v>
       </c>
       <c r="F27" t="n">
-        <v>224.41</v>
+        <v>339.91</v>
       </c>
       <c r="G27" t="n">
-        <v>224.41</v>
+        <v>339.91</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>Ja' Vioun Boyd</t>
+          <t>Isabel Garcia</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>SERVER</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>40</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0.33</v>
+        <v>22.72</v>
+      </c>
+      <c r="F28" t="n">
+        <v>162.43</v>
+      </c>
+      <c r="G28" t="n">
+        <v>162.43</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Jacari Howard</t>
+          <t>J'Elle Longoria</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>SERVER</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>21.83</v>
+        <v>26.11</v>
+      </c>
+      <c r="F29" t="n">
+        <v>79.44</v>
+      </c>
+      <c r="G29" t="n">
+        <v>79.44</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>James Yeomans</t>
+          <t>Ja' Vioun Boyd</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1047,74 +1021,64 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>39.24</v>
+        <v>39.99999999999999</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2.62</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
+          <t>Jacari Howard</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>30.26</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>James Yeomans</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>38.23</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
           <t>Jaykob Elizondo</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>Kitchen</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>35.29</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Jeremiah Wilhelms</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="n">
-        <v>139.65</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>139.65</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Jeremiah Wilhelms</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>10.02</v>
-      </c>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="n">
-        <v>35.38</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>35.38</v>
+      <c r="C33" t="n">
+        <v>40</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1.64</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Jessica Bain</t>
+          <t>Jesus Garza</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1123,7 +1087,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>30.05</v>
+        <v>30.82</v>
       </c>
     </row>
     <row r="35">
@@ -1156,13 +1120,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>14.23</v>
+        <v>13.02</v>
       </c>
       <c r="F36" t="n">
-        <v>103.9</v>
+        <v>88</v>
       </c>
       <c r="G36" t="n">
-        <v>103.9</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37">
@@ -1177,13 +1141,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>26.14</v>
+        <v>18.89</v>
       </c>
       <c r="F37" t="n">
-        <v>374.58</v>
+        <v>109.26</v>
       </c>
       <c r="G37" t="n">
-        <v>374.58</v>
+        <v>109.26</v>
       </c>
     </row>
     <row r="38">
@@ -1198,13 +1162,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>28.63</v>
+        <v>26.11</v>
       </c>
       <c r="F38" t="n">
-        <v>269.74</v>
+        <v>236.71</v>
       </c>
       <c r="G38" t="n">
-        <v>269.74</v>
+        <v>236.71</v>
       </c>
     </row>
     <row r="39">
@@ -1219,55 +1183,59 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>14.57</v>
+        <v>12.83</v>
       </c>
       <c r="F39" t="n">
-        <v>213.96</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>213.96</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Kiara Mccoy</t>
         </is>
       </c>
-      <c r="B40" s="1" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>12.38</v>
-      </c>
-      <c r="F40" t="n">
-        <v>13</v>
-      </c>
-      <c r="G40" t="n">
-        <v>13</v>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>21.14</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>Lariah Saenz</t>
-        </is>
-      </c>
-      <c r="B41" s="1" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>24.75</v>
-      </c>
-      <c r="F41" t="n">
-        <v>299.03</v>
-      </c>
-      <c r="G41" t="n">
-        <v>299.03</v>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Kiara Mccoy</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="n">
+        <v>148.54</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>148.54</v>
       </c>
     </row>
     <row r="42">
@@ -1297,13 +1265,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>18.74</v>
+        <v>23.27</v>
       </c>
       <c r="F43" t="n">
-        <v>124.13</v>
+        <v>191.17</v>
       </c>
       <c r="G43" t="n">
-        <v>124.13</v>
+        <v>191.17</v>
       </c>
     </row>
     <row r="44">
@@ -1325,52 +1293,53 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>34.53</v>
+        <v>8.559999999999999</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Michaela Mireles</t>
         </is>
       </c>
-      <c r="B46" s="1" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
-      <c r="C46" t="n">
-        <v>20.09</v>
-      </c>
-      <c r="F46" t="n">
-        <v>166.8</v>
-      </c>
-      <c r="G46" t="n">
-        <v>166.8</v>
+      <c r="C46" s="3" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="n">
+        <v>254.55</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>254.55</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="inlineStr">
-        <is>
-          <t>Noel Rodriguez</t>
-        </is>
-      </c>
-      <c r="B47" s="1" t="inlineStr">
-        <is>
-          <t>HOST</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>9</v>
-      </c>
-      <c r="E47" t="n">
-        <v>7</v>
-      </c>
-      <c r="F47" t="n">
-        <v>9</v>
-      </c>
-      <c r="G47" t="n">
-        <v>16</v>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Michaela Mireles</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="48">
@@ -1385,85 +1354,101 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>11.98</v>
+        <v>12.92</v>
       </c>
       <c r="F48" t="n">
-        <v>115.37</v>
+        <v>34.74</v>
       </c>
       <c r="G48" t="n">
-        <v>115.37</v>
+        <v>34.74</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>Selena Gomez</t>
+          <t>Selena Cuellar</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>Bar Manager</t>
+          <t>SERVER</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>33.31</v>
+        <v>30.68</v>
       </c>
       <c r="F49" t="n">
-        <v>239.9</v>
+        <v>266.31</v>
       </c>
       <c r="G49" t="n">
-        <v>239.9</v>
+        <v>266.31</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>Sergio Benavente</t>
+          <t>Selena Gomez</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>Busser</t>
+          <t>Bar Manager</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>18.4</v>
+        <v>32.31</v>
+      </c>
+      <c r="F50" t="n">
+        <v>168.61</v>
+      </c>
+      <c r="G50" t="n">
+        <v>168.61</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>Sonya Mendez</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t>Kitchen</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>26.23</v>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Taylor McCarthy</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SERVER</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Taylor McCarthy</t>
         </is>
       </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>SERVER</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>27.43</v>
-      </c>
-      <c r="F52" t="n">
-        <v>188.58</v>
-      </c>
-      <c r="G52" t="n">
-        <v>188.58</v>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="3" t="n">
+        <v>114.41</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>114.41</v>
       </c>
     </row>
     <row r="53">
@@ -1485,28 +1470,28 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1045.65</v>
+        <v>1089.54</v>
       </c>
       <c r="C54" t="n">
-        <v>1018.59</v>
+        <v>1048.39</v>
       </c>
       <c r="D54" t="n">
-        <v>27.06000000000001</v>
+        <v>41.15000000000001</v>
       </c>
       <c r="E54" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F54" t="n">
-        <v>5720.120000000001</v>
+        <v>4592</v>
       </c>
       <c r="G54" t="n">
-        <v>5727.120000000001</v>
+        <v>4602</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>Total hours for the BHB Kingsville for the week is 1045.65 of which 27.06 or 2.59% is considered overtime.</t>
+          <t>Total hours for the BHB Kingsville for the week is 1089.54 of which 41.15 or 3.78% is considered overtime.</t>
         </is>
       </c>
     </row>

</xml_diff>